<commit_message>
conch1.5: re-extract TCGA five-crop at 256 px and recompute its results
The TCGA CONCH v1.5 five-crop features mixed 224 px and 256 px crops between
slides. 182 slides were re-extracted with FiveCrop(256) into
dataset/Features/Conch_v1_5_fivecrop_256 (fp32, as the baseline), verified, and
the Conch1_5 rows of TCGA_Results, TCGA_FULL_Models and TCGA_PAIP_EV_Results
recomputed with the published runners; experiments/final_analysis/results
regenerated. Only the Conch1_5 entries of the control files changed.
TCGA-CV +0.008 to +0.013 AUROC for Conch1_5; headline claims unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/slide_classification/TCGA_Results/Averaging/Conch1_5/1-MSIH/Output/cross_valid_avg_eval_metrics.xlsx
+++ b/slide_classification/TCGA_Results/Averaging/Conch1_5/1-MSIH/Output/cross_valid_avg_eval_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="baseline" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="baseline" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -468,19 +468,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.883495145631068</v>
+        <v>0.8349514563106796</v>
       </c>
       <c r="C2" t="n">
-        <v>0.8865979381443299</v>
+        <v>0.865979381443299</v>
       </c>
       <c r="D2" t="n">
-        <v>0.8392857142857143</v>
+        <v>0.8482142857142857</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8910891089108911</v>
+        <v>0.8712871287128713</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8751169767430008</v>
+        <v>0.8551080630452839</v>
       </c>
     </row>
     <row r="3">
@@ -490,19 +490,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.7106060606060607</v>
+        <v>0.6268939393939393</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7394688644688645</v>
+        <v>0.6625457875457875</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6673913043478261</v>
+        <v>0.6728260869565217</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7219101123595506</v>
+        <v>0.674625468164794</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7098440854455754</v>
+        <v>0.6592228205152606</v>
       </c>
     </row>
     <row r="4">
@@ -512,19 +512,19 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.7358974358974359</v>
+        <v>0.6376991516656321</v>
       </c>
       <c r="C4" t="n">
-        <v>0.7474556213017751</v>
+        <v>0.6793796084413933</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6879256965944273</v>
+        <v>0.6979216246231953</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7301433082341511</v>
+        <v>0.6810784551858149</v>
       </c>
       <c r="F4" t="n">
-        <v>0.7253555155069473</v>
+        <v>0.6740197099790088</v>
       </c>
     </row>
     <row r="5">
@@ -534,19 +534,19 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.8758277321384118</v>
+        <v>0.8271651811273225</v>
       </c>
       <c r="C5" t="n">
-        <v>0.884665405965961</v>
+        <v>0.8584145257810595</v>
       </c>
       <c r="D5" t="n">
-        <v>0.8276426360017691</v>
+        <v>0.8348972144783663</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8890257012099073</v>
+        <v>0.8688485559753449</v>
       </c>
       <c r="F5" t="n">
-        <v>0.8692903688290122</v>
+        <v>0.8473313693405233</v>
       </c>
     </row>
     <row r="6">
@@ -556,19 +556,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.8143939393939394</v>
+        <v>0.8128787878787879</v>
       </c>
       <c r="C6" t="n">
-        <v>0.8113553113553114</v>
+        <v>0.8003663003663004</v>
       </c>
       <c r="D6" t="n">
-        <v>0.7119565217391305</v>
+        <v>0.7369565217391304</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6367041198501873</v>
+        <v>0.6301498127340824</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7436024730846422</v>
+        <v>0.7450878556795753</v>
       </c>
     </row>
     <row r="7">
@@ -579,27 +579,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[[84, 4], [8, 7]]</t>
+          <t>[[81, 7], [10, 5]]</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>[[79, 5], [6, 7]]</t>
+          <t>[[79, 5], [8, 5]]</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>[[86, 6], [12, 8]]</t>
+          <t>[[87, 5], [12, 8]]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[[84, 5], [6, 6]]</t>
+          <t>[[83, 6], [7, 5]]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[[83, 5], [8, 7]]</t>
+          <t>[[82, 6], [9, 6]]</t>
         </is>
       </c>
     </row>
@@ -610,19 +610,19 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.8446601941747572</v>
+        <v>0.7766990291262136</v>
       </c>
       <c r="C8" t="n">
-        <v>0.7628865979381443</v>
+        <v>0.7010309278350515</v>
       </c>
       <c r="D8" t="n">
-        <v>0.7589285714285714</v>
+        <v>0.6428571428571429</v>
       </c>
       <c r="E8" t="n">
-        <v>0.8217821782178217</v>
+        <v>0.8118811881188119</v>
       </c>
       <c r="F8" t="n">
-        <v>0.7970643854398236</v>
+        <v>0.733117071984305</v>
       </c>
     </row>
     <row r="9">
@@ -632,19 +632,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.7708333333333333</v>
+        <v>0.7587121212121212</v>
       </c>
       <c r="C9" t="n">
-        <v>0.603021978021978</v>
+        <v>0.6973443223443223</v>
       </c>
       <c r="D9" t="n">
-        <v>0.6967391304347825</v>
+        <v>0.7043478260869566</v>
       </c>
       <c r="E9" t="n">
-        <v>0.6465355805243446</v>
+        <v>0.6769662921348314</v>
       </c>
       <c r="F9" t="n">
-        <v>0.6792825055786096</v>
+        <v>0.7093426404445577</v>
       </c>
     </row>
     <row r="10">
@@ -654,19 +654,19 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.7307189542483661</v>
+        <v>0.673015873015873</v>
       </c>
       <c r="C10" t="n">
-        <v>0.5800865800865801</v>
+        <v>0.5928499059198147</v>
       </c>
       <c r="D10" t="n">
-        <v>0.657259435566134</v>
+        <v>0.5906432748538011</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6268472906403941</v>
+        <v>0.6379928315412187</v>
       </c>
       <c r="F10" t="n">
-        <v>0.6487280651353686</v>
+        <v>0.6236254713326769</v>
       </c>
     </row>
     <row r="11">
@@ -676,19 +676,19 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.8548638873024937</v>
+        <v>0.8035136384650947</v>
       </c>
       <c r="C11" t="n">
-        <v>0.7828803498906591</v>
+        <v>0.746466957039451</v>
       </c>
       <c r="D11" t="n">
-        <v>0.7772623500267158</v>
+        <v>0.6846282372598161</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8324635419206945</v>
+        <v>0.8292700237765711</v>
       </c>
       <c r="F11" t="n">
-        <v>0.8118675322851407</v>
+        <v>0.7659697141352333</v>
       </c>
     </row>
     <row r="12">
@@ -698,19 +698,19 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.7856060606060606</v>
+        <v>0.8212121212121213</v>
       </c>
       <c r="C12" t="n">
-        <v>0.6501831501831502</v>
+        <v>0.7371794871794872</v>
       </c>
       <c r="D12" t="n">
-        <v>0.753804347826087</v>
+        <v>0.7842391304347825</v>
       </c>
       <c r="E12" t="n">
-        <v>0.6891385767790262</v>
+        <v>0.7209737827715356</v>
       </c>
       <c r="F12" t="n">
-        <v>0.7196830338485809</v>
+        <v>0.7659011303994816</v>
       </c>
     </row>
     <row r="13">
@@ -721,27 +721,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[[77, 11], [5, 10]]</t>
+          <t>[[69, 19], [4, 11]]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>[[69, 15], [8, 5]]</t>
+          <t>[[59, 25], [4, 9]]</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>[[73, 19], [8, 12]]</t>
+          <t>[[56, 36], [4, 16]]</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>[[78, 11], [7, 5]]</t>
+          <t>[[76, 13], [6, 6]]</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[[74, 14], [7, 8]]</t>
+          <t>[[65, 23], [4, 10]]</t>
         </is>
       </c>
     </row>
@@ -755,16 +755,16 @@
         <v>0.8737864077669902</v>
       </c>
       <c r="C14" t="n">
-        <v>0.865979381443299</v>
+        <v>0.8762886597938144</v>
       </c>
       <c r="D14" t="n">
-        <v>0.8571428571428571</v>
+        <v>0.8482142857142857</v>
       </c>
       <c r="E14" t="n">
         <v>0.8910891089108911</v>
       </c>
       <c r="F14" t="n">
-        <v>0.8719994388160094</v>
+        <v>0.8723446155464953</v>
       </c>
     </row>
     <row r="15">
@@ -774,19 +774,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.6496212121212122</v>
+        <v>0.6772727272727272</v>
       </c>
       <c r="C15" t="n">
-        <v>0.5325091575091575</v>
+        <v>0.5384615384615384</v>
       </c>
       <c r="D15" t="n">
-        <v>0.6195652173913043</v>
+        <v>0.5945652173913043</v>
       </c>
       <c r="E15" t="n">
         <v>0.5777153558052435</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5948527357067294</v>
+        <v>0.5970037097327033</v>
       </c>
     </row>
     <row r="16">
@@ -796,19 +796,19 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.681872178664766</v>
+        <v>0.7040883977900552</v>
       </c>
       <c r="C16" t="n">
-        <v>0.5303538175046555</v>
+        <v>0.5380952380952381</v>
       </c>
       <c r="D16" t="n">
-        <v>0.651903651903652</v>
+        <v>0.617286432160804</v>
       </c>
       <c r="E16" t="n">
         <v>0.6039215686274509</v>
       </c>
       <c r="F16" t="n">
-        <v>0.6170128041751312</v>
+        <v>0.6158479091683871</v>
       </c>
     </row>
     <row r="17">
@@ -818,19 +818,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.8569939127205457</v>
+        <v>0.8629083302043663</v>
       </c>
       <c r="C17" t="n">
-        <v>0.8209564399393345</v>
+        <v>0.8273932253313697</v>
       </c>
       <c r="D17" t="n">
-        <v>0.8237318237318237</v>
+        <v>0.8083991385498923</v>
       </c>
       <c r="E17" t="n">
         <v>0.8610366919044846</v>
       </c>
       <c r="F17" t="n">
-        <v>0.8406797170740472</v>
+        <v>0.8399343464975283</v>
       </c>
     </row>
     <row r="18">
@@ -840,19 +840,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.7708333333333334</v>
+        <v>0.8113636363636364</v>
       </c>
       <c r="C18" t="n">
-        <v>0.6886446886446888</v>
+        <v>0.7188644688644689</v>
       </c>
       <c r="D18" t="n">
-        <v>0.7190217391304348</v>
+        <v>0.7173913043478262</v>
       </c>
       <c r="E18" t="n">
         <v>0.7045880149812734</v>
       </c>
       <c r="F18" t="n">
-        <v>0.7207719440224325</v>
+        <v>0.7380518561393012</v>
       </c>
     </row>
     <row r="19">
@@ -863,17 +863,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[[85, 3], [10, 5]]</t>
+          <t>[[84, 4], [9, 6]]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>[[83, 1], [12, 1]]</t>
+          <t>[[84, 0], [12, 1]]</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>[[91, 1], [15, 5]]</t>
+          <t>[[91, 1], [16, 4]]</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -894,19 +894,19 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.6019417475728155</v>
+        <v>0.6213592233009708</v>
       </c>
       <c r="C20" t="n">
-        <v>0.3814432989690721</v>
+        <v>0.4123711340206185</v>
       </c>
       <c r="D20" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.6339285714285714</v>
       </c>
       <c r="E20" t="n">
         <v>0.7821782178217822</v>
       </c>
       <c r="F20" t="n">
-        <v>0.6021051018052033</v>
+        <v>0.6124592866429858</v>
       </c>
     </row>
     <row r="21">
@@ -916,19 +916,19 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.656439393939394</v>
+        <v>0.6401515151515151</v>
       </c>
       <c r="C21" t="n">
-        <v>0.4152930402930403</v>
+        <v>0.4331501831501832</v>
       </c>
       <c r="D21" t="n">
-        <v>0.6260869565217391</v>
+        <v>0.6010869565217392</v>
       </c>
       <c r="E21" t="n">
         <v>0.6961610486891385</v>
       </c>
       <c r="F21" t="n">
-        <v>0.598495109860828</v>
+        <v>0.5926374258781439</v>
       </c>
     </row>
     <row r="22">
@@ -938,19 +938,19 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.5312465312465313</v>
+        <v>0.536838464199239</v>
       </c>
       <c r="C22" t="n">
-        <v>0.337431693989071</v>
+        <v>0.3589565217391305</v>
       </c>
       <c r="D22" t="n">
-        <v>0.5625</v>
+        <v>0.5472739820565907</v>
       </c>
       <c r="E22" t="n">
         <v>0.6281793842034806</v>
       </c>
       <c r="F22" t="n">
-        <v>0.5148394023597707</v>
+        <v>0.5178120880496102</v>
       </c>
     </row>
     <row r="23">
@@ -960,19 +960,19 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.6602653010420001</v>
+        <v>0.6770660872543851</v>
       </c>
       <c r="C23" t="n">
-        <v>0.4624246521322742</v>
+        <v>0.4944007171671896</v>
       </c>
       <c r="D23" t="n">
-        <v>0.6830357142857143</v>
+        <v>0.6746031746031746</v>
       </c>
       <c r="E23" t="n">
         <v>0.8106087717205457</v>
       </c>
       <c r="F23" t="n">
-        <v>0.6540836097951337</v>
+        <v>0.6641696876863238</v>
       </c>
     </row>
     <row r="24">
@@ -982,19 +982,19 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.7416666666666667</v>
+        <v>0.7553030303030303</v>
       </c>
       <c r="C24" t="n">
-        <v>0.4908424908424909</v>
+        <v>0.5210622710622711</v>
       </c>
       <c r="D24" t="n">
-        <v>0.6722826086956523</v>
+        <v>0.6777173913043478</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6956928838951311</v>
+        <v>0.6919475655430711</v>
       </c>
       <c r="F24" t="n">
-        <v>0.6501211625249852</v>
+        <v>0.66150756455318</v>
       </c>
     </row>
     <row r="25">
@@ -1005,17 +1005,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>[[51, 37], [4, 11]]</t>
+          <t>[[54, 34], [5, 10]]</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>[[31, 53], [7, 6]]</t>
+          <t>[[34, 50], [7, 6]]</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>[[60, 32], [8, 12]]</t>
+          <t>[[60, 32], [9, 11]]</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>[[54, 35], [6, 9]]</t>
+          <t>[[55, 33], [6, 8]]</t>
         </is>
       </c>
     </row>
@@ -1036,19 +1036,19 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.883495145631068</v>
+        <v>0.8737864077669902</v>
       </c>
       <c r="C26" t="n">
-        <v>0.8969072164948454</v>
+        <v>0.9072164948453608</v>
       </c>
       <c r="D26" t="n">
-        <v>0.8392857142857143</v>
+        <v>0.8303571428571429</v>
       </c>
       <c r="E26" t="n">
-        <v>0.8514851485148515</v>
+        <v>0.8613861386138614</v>
       </c>
       <c r="F26" t="n">
-        <v>0.8677933062316198</v>
+        <v>0.8681865460208388</v>
       </c>
     </row>
     <row r="27">
@@ -1058,19 +1058,19 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.7659090909090909</v>
+        <v>0.7325757575757575</v>
       </c>
       <c r="C27" t="n">
-        <v>0.6478937728937729</v>
+        <v>0.6538461538461539</v>
       </c>
       <c r="D27" t="n">
-        <v>0.6086956521739131</v>
+        <v>0.6032608695652174</v>
       </c>
       <c r="E27" t="n">
-        <v>0.5552434456928839</v>
+        <v>0.5608614232209738</v>
       </c>
       <c r="F27" t="n">
-        <v>0.6444354904174152</v>
+        <v>0.6376360510520257</v>
       </c>
     </row>
     <row r="28">
@@ -1080,19 +1080,19 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>0.7659090909090909</v>
+        <v>0.7391389051237094</v>
       </c>
       <c r="C28" t="n">
-        <v>0.6938131313131313</v>
+        <v>0.7098703888334995</v>
       </c>
       <c r="D28" t="n">
-        <v>0.6326530612244898</v>
+        <v>0.6236958443854996</v>
       </c>
       <c r="E28" t="n">
-        <v>0.5642795513373597</v>
+        <v>0.5730676328502415</v>
       </c>
       <c r="F28" t="n">
-        <v>0.6641637086960179</v>
+        <v>0.6614431927982376</v>
       </c>
     </row>
     <row r="29">
@@ -1102,19 +1102,19 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.883495145631068</v>
+        <v>0.8719668469204596</v>
       </c>
       <c r="C29" t="n">
-        <v>0.8763407268561908</v>
+        <v>0.8850150579190263</v>
       </c>
       <c r="D29" t="n">
-        <v>0.8097667638483965</v>
+        <v>0.8029682960717445</v>
       </c>
       <c r="E29" t="n">
-        <v>0.8339726121015899</v>
+        <v>0.840543836992395</v>
       </c>
       <c r="F29" t="n">
-        <v>0.8508938121093113</v>
+        <v>0.8501235094759063</v>
       </c>
     </row>
     <row r="30">
@@ -1124,19 +1124,19 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.8825757575757576</v>
+        <v>0.8795454545454545</v>
       </c>
       <c r="C30" t="n">
-        <v>0.8076923076923077</v>
+        <v>0.771978021978022</v>
       </c>
       <c r="D30" t="n">
-        <v>0.7331521739130435</v>
+        <v>0.7353260869565218</v>
       </c>
       <c r="E30" t="n">
-        <v>0.7350187265917603</v>
+        <v>0.75</v>
       </c>
       <c r="F30" t="n">
-        <v>0.7896097414432173</v>
+        <v>0.7842123908699996</v>
       </c>
     </row>
     <row r="31">
@@ -1147,27 +1147,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>[[82, 6], [6, 9]]</t>
+          <t>[[82, 6], [7, 8]]</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>[[83, 1], [9, 4]]</t>
+          <t>[[84, 0], [9, 4]]</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>[[89, 3], [15, 5]]</t>
+          <t>[[88, 4], [15, 5]]</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>[[84, 5], [10, 2]]</t>
+          <t>[[85, 4], [10, 2]]</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>[[84, 4], [10, 5]]</t>
+          <t>[[85, 4], [10, 5]]</t>
         </is>
       </c>
     </row>
@@ -1290,38 +1290,38 @@
         <v>413</v>
       </c>
       <c r="F2" t="n">
-        <v>0.8751169767430008</v>
+        <v>0.8551080630452839</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0208626134741509</v>
+        <v>0.01443745727725287</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7098440854455754</v>
+        <v>0.6592228205152606</v>
       </c>
       <c r="I2" t="n">
-        <v>0.02658023592232629</v>
+        <v>0.01922556291068032</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7253555155069473</v>
+        <v>0.6740197099790088</v>
       </c>
       <c r="K2" t="n">
-        <v>0.02249144873437842</v>
+        <v>0.02218692675470769</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8692903688290122</v>
+        <v>0.8473313693405233</v>
       </c>
       <c r="M2" t="n">
-        <v>0.02451094592134026</v>
+        <v>0.01693449904447639</v>
       </c>
       <c r="N2" t="n">
-        <v>0.7436024730846422</v>
+        <v>0.7450878556795753</v>
       </c>
       <c r="O2" t="n">
-        <v>0.07421354821855747</v>
+        <v>0.07233289231603517</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>[[83, 5], [8, 7]]</t>
+          <t>[[82, 6], [9, 6]]</t>
         </is>
       </c>
     </row>
@@ -1348,38 +1348,38 @@
         <v>413</v>
       </c>
       <c r="F3" t="n">
-        <v>0.7970643854398236</v>
+        <v>0.733117071984305</v>
       </c>
       <c r="G3" t="n">
-        <v>0.03707691922800224</v>
+        <v>0.06572584809490147</v>
       </c>
       <c r="H3" t="n">
-        <v>0.6792825055786096</v>
+        <v>0.7093426404445577</v>
       </c>
       <c r="I3" t="n">
-        <v>0.06239855162115074</v>
+        <v>0.03022615328168998</v>
       </c>
       <c r="J3" t="n">
-        <v>0.6487280651353686</v>
+        <v>0.6236254713326769</v>
       </c>
       <c r="K3" t="n">
-        <v>0.05473963815456256</v>
+        <v>0.03420816250853725</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8118675322851407</v>
+        <v>0.7659697141352333</v>
       </c>
       <c r="M3" t="n">
-        <v>0.03282779896671353</v>
+        <v>0.05570742510964476</v>
       </c>
       <c r="N3" t="n">
-        <v>0.7196830338485809</v>
+        <v>0.7659011303994816</v>
       </c>
       <c r="O3" t="n">
-        <v>0.05308791578975674</v>
+        <v>0.03949363019560739</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>[[74, 14], [7, 8]]</t>
+          <t>[[65, 23], [4, 10]]</t>
         </is>
       </c>
     </row>
@@ -1406,34 +1406,34 @@
         <v>413</v>
       </c>
       <c r="F4" t="n">
-        <v>0.8719994388160094</v>
+        <v>0.8723446155464953</v>
       </c>
       <c r="G4" t="n">
-        <v>0.01249567797425334</v>
+        <v>0.01542127669107679</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5948527357067294</v>
+        <v>0.5970037097327033</v>
       </c>
       <c r="I4" t="n">
-        <v>0.04413248319588085</v>
+        <v>0.0506169137643562</v>
       </c>
       <c r="J4" t="n">
-        <v>0.6170128041751312</v>
+        <v>0.6158479091683871</v>
       </c>
       <c r="K4" t="n">
-        <v>0.05723912589592902</v>
+        <v>0.05911042344269352</v>
       </c>
       <c r="L4" t="n">
-        <v>0.8406797170740472</v>
+        <v>0.8399343464975283</v>
       </c>
       <c r="M4" t="n">
-        <v>0.01841737056090903</v>
+        <v>0.02304811255526937</v>
       </c>
       <c r="N4" t="n">
-        <v>0.7207719440224325</v>
+        <v>0.7380518561393012</v>
       </c>
       <c r="O4" t="n">
-        <v>0.0308353936824941</v>
+        <v>0.0426891672894704</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -1464,38 +1464,38 @@
         <v>413</v>
       </c>
       <c r="F5" t="n">
-        <v>0.6021051018052033</v>
+        <v>0.6124592866429858</v>
       </c>
       <c r="G5" t="n">
-        <v>0.1438564509131552</v>
+        <v>0.1317003449900811</v>
       </c>
       <c r="H5" t="n">
-        <v>0.598495109860828</v>
+        <v>0.5926374258781439</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1086513736230157</v>
+        <v>0.09808453537695876</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5148394023597707</v>
+        <v>0.5178120880496102</v>
       </c>
       <c r="K5" t="n">
-        <v>0.108236053281019</v>
+        <v>0.09829297685491711</v>
       </c>
       <c r="L5" t="n">
-        <v>0.6540836097951337</v>
+        <v>0.6641696876863238</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1246091088457173</v>
+        <v>0.1124067207231976</v>
       </c>
       <c r="N5" t="n">
-        <v>0.6501211625249852</v>
+        <v>0.66150756455318</v>
       </c>
       <c r="O5" t="n">
-        <v>0.0952866544518539</v>
+        <v>0.0861855875459266</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>[[54, 35], [6, 9]]</t>
+          <t>[[55, 33], [6, 8]]</t>
         </is>
       </c>
     </row>
@@ -1522,38 +1522,38 @@
         <v>413</v>
       </c>
       <c r="F6" t="n">
-        <v>0.8677933062316198</v>
+        <v>0.8681865460208388</v>
       </c>
       <c r="G6" t="n">
-        <v>0.02330668540360503</v>
+        <v>0.02753182086896513</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6444354904174152</v>
+        <v>0.6376360510520257</v>
       </c>
       <c r="I6" t="n">
-        <v>0.07746023530481946</v>
+        <v>0.06393807920217824</v>
       </c>
       <c r="J6" t="n">
-        <v>0.6641637086960179</v>
+        <v>0.6614431927982376</v>
       </c>
       <c r="K6" t="n">
-        <v>0.07449996117203116</v>
+        <v>0.06636437097176962</v>
       </c>
       <c r="L6" t="n">
-        <v>0.8508938121093113</v>
+        <v>0.8501235094759063</v>
       </c>
       <c r="M6" t="n">
-        <v>0.03036508490803498</v>
+        <v>0.03166202701801719</v>
       </c>
       <c r="N6" t="n">
-        <v>0.7896097414432173</v>
+        <v>0.7842123908699996</v>
       </c>
       <c r="O6" t="n">
-        <v>0.06151685783515892</v>
+        <v>0.05656507582266614</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>[[84, 4], [10, 5]]</t>
+          <t>[[85, 4], [10, 5]]</t>
         </is>
       </c>
     </row>

</xml_diff>